<commit_message>
new readme for entrypoint
</commit_message>
<xml_diff>
--- a/out/test_data.xlsx
+++ b/out/test_data.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,11 @@
           <t>Code (4,2)</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Code (3,2)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -581,6 +586,9 @@
       <c r="P3" t="n">
         <v>6</v>
       </c>
+      <c r="Q3" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -631,6 +639,9 @@
         <v>72</v>
       </c>
       <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>